<commit_message>
done ai log week 2
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenHoHongNam.xlsx
+++ b/AI Audit Log_NguyenHoHongNam.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\ai-audit-log-123-NguyenHoHongNam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B7416E5-F09C-44F2-ADB1-EFDC294D910B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6553BE0B-48F2-4E4D-A4B6-A4D839B44123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
-    <sheet name="Assignment 1" sheetId="2" r:id="rId2"/>
-    <sheet name="Assignment 2" sheetId="3" r:id="rId3"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week1" sheetId="3" r:id="rId2"/>
+    <sheet name="Week2" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="37">
   <si>
     <t>Nội dung Prompt (Câu lệnh)</t>
   </si>
@@ -89,6 +88,76 @@
   <si>
     <t>Phản hồi: AI đưa ra SDLC chuẩn: Khảo sát yêu cầu -&gt; Phân tích -&gt; Thiết kế -&gt; Lập trình -&gt; Kiểm thử -&gt; Triển khai -&gt; Bảo trì.
 Kiểm chứng: Nhóm quyết định dồn nhiều nguồn lực và thời gian nhất vào giai đoạn Thiết kế cơ sở dữ liệu và Kiểm thử (Testing), vì đây là phần dễ phát sinh lỗi logic nhất khi làm web.</t>
+  </si>
+  <si>
+    <t>Khái niệm &amp; Bản chất của Use Case</t>
+  </si>
+  <si>
+    <t>"Tôi đang học về kỹ nghệ phần mềm. Hãy giải thích rõ Use Case là gì, mục đích sử dụng và các thành phần cốt lõi cấu thành một Use Case chuẩn."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI định nghĩa Use Case là chuỗi các bước tương tác giữa Tác nhân (Actor) và Hệ thống để đạt được một mục tiêu cụ thể. Thành phần gồm: Actor, Goal, Pre-conditions, Post-conditions, và Main Flow.
+Quyết định: Nhận thức rõ Use Case dùng để làm rõ hệ thống làm gì (What) chứ không phải hệ thống làm như thế nào (How). Tập trung vào việc xác định rõ ranh giới hệ thống (System Boundary) để tránh viết lan man sang phần giao</t>
+  </si>
+  <si>
+    <t>Xác định và Phân rã Use Case</t>
+  </si>
+  <si>
+    <t>"Tôi đang làm app [tìm việc/đặt đồ ăn]. Hãy gợi ý danh sách các Use Case chính và cách phân tách chúng bằng quan hệ &lt;&lt;include&gt;&gt; và &lt;&lt;extend&gt;&gt;."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI liệt kê danh sách tính năng dày đặc và đề xuất lồng ghép nhiều quan hệ &lt;&lt;include&gt;&gt;, &lt;&lt;extend&gt;&gt; để tái sử dụng kịch bản.
+Quyết định: Nhóm quyết định giữ sơ đồ ở mức tổng quan (High-level). Chỉ dùng &lt;&lt;include&gt;&gt; cho các tác vụ lặp lại bắt buộc (như Đăng nhập, Xác thực) và &lt;&lt;extend&gt;&gt; cho tính năng tùy chọn (như Áp mã giảm giá), tránh phân rã quá sâu làm sơ đồ bị rối mắt, khó đọc.</t>
+  </si>
+  <si>
+    <t>Tối ưu hóa Kịch bản Use Case (Use Case Specification)</t>
+  </si>
+  <si>
+    <t>"Làm sao để tối ưu hóa và viết một kịch bản mô tả chi tiết Use Case (Main Flow &amp; Alternative Flow) ngắn gọn, dễ hiểu cho cả Dev và Tester?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đưa ra một template kịch bản rất dài dòng, mô tả chi tiết từng click chuột của người dùng và từng dòng thông báo hiển thị của hệ thống.
+Quyết định: Tối ưu hóa bằng cách lược bỏ các yếu tố giao diện (UI-independent). Thay vì viết "Người dùng click nút Đăng ký", đổi thành "Người dùng chọn xác nhận đăng ký". Giữ số lượng bước trong luồng chính (Main Flow) từ 5-9 bước. Đưa các trường hợp lỗi, ngoại lệ vào Luồng thay thế (Alternative Flow) để kịch bản mạch lạc hơn.</t>
+  </si>
+  <si>
+    <t>Tối ưu hóa để Chuyển đổi sang Thiết kế &amp; Testing</t>
+  </si>
+  <si>
+    <t>"Lập biểu đồ Use Case xong thì làm gì tiếp theo? Hãy hướng dẫn cách tối ưu Use Case để phục vụ tốt nhất cho việc thiết kế Database và viết Test Case."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất quy trình chuẩn: Từ Use Case vẽ Sequence Diagram -&gt; Thiết kế Class -&gt; Tạo ERD (Database) -&gt; Viết Test Case cho từng luồng.
+Quyết định: Nhóm quyết định tối ưu bằng cách tận dụng các Post-conditions (Điều kiện sau) của Use Case để định hình các bảng dữ liệu trong ERD. Đồng thời, biến trực tiếp các luồng tương tác (Main/Alternative Flow) thành các kịch bản kiểm thử (Test Scenario) lõi, giúp Tester không bị sót các trường hợp kiểm thử quan trọng.</t>
+  </si>
+  <si>
+    <t>Quản lý ma trận truy vết (Traceability Matrix)</t>
+  </si>
+  <si>
+    <t>"Làm sao để đảm bảo các Use Case đã bao phủ toàn bộ yêu cầu (Requirements) ban đầu của khách hàng và không bị sót tính năng?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI hướng dẫn xây dựng một ma trận truy vết (Traceability Matrix) khổng lồ bằng Excel để ánh xạ thủ công từng dòng Requirement sang từng Use Case tương ứng.
+Quyết định: Nhóm quyết định không sa đà vào việc làm ma trận quá chi tiết cho mọi tính năng nhỏ lẻ để tránh tốn thời gian. Thay vào đó, nhóm chỉ tập trung ánh xạ các Functional Requirements cốt lõi của dự án vào các Use Case chính, đảm bảo mỗi Requirement có ít nhất một Use Case giải quyết.</t>
+  </si>
+  <si>
+    <t>Tối ưu hóa Use Case cho kiến trúc phân tầng</t>
+  </si>
+  <si>
+    <t>"Tôi muốn thiết kế hệ thống theo mô hình Clean Architecture / Repository Pattern. Tôi nên áp dụng Use Case vào code như thế nào để tối ưu?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích khái niệm Use Case trong Clean Architecture (Application Business Rules) và đề xuất viết mỗi Use Case thành một class/file xử lý logic độc lập (Single Responsibility).
+Quyết định: Nhóm quyết định áp dụng triệt để tư duy này vào dự án. Tách biệt hoàn toàn logic nghiệp vụ trong Use Case ra khỏi Controller (Frontend/API) và Repository (Database). Điều này giúp code cực kỳ tường minh, dễ viết Unit Test độc lập và dễ bảo trì khi hệ thống phình to.</t>
+  </si>
+  <si>
+    <t>Xử lý Non-Functional Requirements (Yêu cầu phi chức năng)</t>
+  </si>
+  <si>
+    <t>"Các yêu cầu về bảo mật (Security), hiệu năng (Performance) có nên đưa vào sơ đồ hoặc kịch bản Use Case không? Hãy gợi ý cách làm."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất tạo thêm các Use Case đặc biệt cho bảo mật hoặc viết lồng ghép các tiêu chí hiệu năng (ví dụ: phản hồi &lt; 2s) vào từng bước của kịch bản Use Case.
+Quyết định: Nhóm quyết định giữ Use Case thuần túy tập trung vào chức năng để tránh làm rối kịch bản. Các yêu cầu phi chức năng (như bảo mật, hiệu năng) sẽ được tách riêng ra thành một mục "Special Requirements" (Yêu cầu đặc biệt) đính kèm ở phần cuối của tài liệu mô tả Use Case đó.</t>
   </si>
 </sst>
 </file>
@@ -148,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -170,6 +239,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -591,28 +684,213 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E3EFE9-6FFB-49CC-BE69-0C0E36C6253E}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="26.88671875" customWidth="1"/>
+    <col min="3" max="3" width="27.109375" customWidth="1"/>
+    <col min="4" max="4" width="55.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="10">
+        <v>1</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="10">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="10">
+        <v>3</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A5" s="10">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="29.88671875" customWidth="1"/>
+    <col min="3" max="3" width="45.109375" customWidth="1"/>
+    <col min="4" max="4" width="81.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="13" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="13" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="13" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A6" s="14">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="14">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A8" s="14">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>